<commit_message>
merge forecast and add people tab
</commit_message>
<xml_diff>
--- a/Expenses.xlsx
+++ b/Expenses.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\ACPL-Automation\ACPL-automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C19FA33C-9B41-4766-97A9-119756869714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26FFFBF6-4B25-4F0B-8D2E-BE1FF02A91D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3720" yWindow="2700" windowWidth="32640" windowHeight="15645" xr2:uid="{3C6E0B95-FFD8-4D7A-85DA-AFCE7993F548}"/>
+    <workbookView xWindow="4605" yWindow="2610" windowWidth="32640" windowHeight="15645" xr2:uid="{3C6E0B95-FFD8-4D7A-85DA-AFCE7993F548}"/>
   </bookViews>
   <sheets>
     <sheet name="Expenses" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="40">
   <si>
     <t>Accounting / Payment Services</t>
   </si>
@@ -99,10 +99,52 @@
     <t>expense_type</t>
   </si>
   <si>
-    <t>Once_accept</t>
-  </si>
-  <si>
     <t>Other</t>
+  </si>
+  <si>
+    <t>6602.09.04</t>
+  </si>
+  <si>
+    <t>Airfare - International</t>
+  </si>
+  <si>
+    <t>Airfare - Domestic</t>
+  </si>
+  <si>
+    <t>6602.09.01</t>
+  </si>
+  <si>
+    <t>Hotels</t>
+  </si>
+  <si>
+    <t>6602.09.03</t>
+  </si>
+  <si>
+    <t>Ground transportation</t>
+  </si>
+  <si>
+    <t>6602.09.02</t>
+  </si>
+  <si>
+    <t>Meals</t>
+  </si>
+  <si>
+    <t>6602.06</t>
+  </si>
+  <si>
+    <t>Entertainment</t>
+  </si>
+  <si>
+    <t>6602.09.99</t>
+  </si>
+  <si>
+    <t>Other personal reimbursement</t>
+  </si>
+  <si>
+    <t>支付的其他与经营活动有关的现金（员工报销）</t>
+  </si>
+  <si>
+    <t>T&amp;E</t>
   </si>
 </sst>
 </file>
@@ -503,14 +545,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{613BF285-6D0C-4CA1-8B6D-EEB5124F663C}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="27.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="43" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>20</v>
       </c>
@@ -523,11 +565,8 @@
       <c r="D1" t="s">
         <v>23</v>
       </c>
-      <c r="E1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -538,10 +577,10 @@
         <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -552,10 +591,10 @@
         <v>19</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -566,10 +605,10 @@
         <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -580,10 +619,10 @@
         <v>19</v>
       </c>
       <c r="D5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>13</v>
       </c>
@@ -594,10 +633,10 @@
         <v>19</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>14</v>
       </c>
@@ -608,10 +647,10 @@
         <v>19</v>
       </c>
       <c r="D7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
@@ -622,10 +661,10 @@
         <v>19</v>
       </c>
       <c r="D8" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
@@ -636,10 +675,10 @@
         <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>17</v>
       </c>
@@ -650,10 +689,10 @@
         <v>19</v>
       </c>
       <c r="D10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>18</v>
       </c>
@@ -664,7 +703,105 @@
         <v>19</v>
       </c>
       <c r="D11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
         <v>25</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" t="s">
+        <v>38</v>
+      </c>
+      <c r="D18" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>